<commit_message>
Final Sim Run Updates
RE-run of simulation due to incorrectly-entered watershed area for the South Thompson Summer 1.3s
</commit_message>
<xml_diff>
--- a/data/CN1.3_watershed_areas.xlsx
+++ b/data/CN1.3_watershed_areas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BAILEYCO\Documents\GitHub\FIA-CN-FSRR-FSAR\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5BDAC2B-E04B-4D62-A86F-E715696C6679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16451147-E59D-4B6D-B772-07EE67BEF293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CAC3600-14F7-4FC2-A03F-D03767E6DF51}"/>
+    <workbookView xWindow="28680" yWindow="-2115" windowWidth="29040" windowHeight="15720" xr2:uid="{6CAC3600-14F7-4FC2-A03F-D03767E6DF51}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -582,7 +582,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>59.7</v>
+        <v>761.7</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>